<commit_message>
Cập nhật lại Testcase
</commit_message>
<xml_diff>
--- a/Test Project/TestUI/document/Nguyen Ba Thinh.xlsx
+++ b/Test Project/TestUI/document/Nguyen Ba Thinh.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="Test Scenario" sheetId="1" r:id="rId1"/>
     <sheet name="Test data" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
+    <sheet name="Testcase" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="144525"/>
 </workbook>
@@ -106,6 +106,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF444746"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>Unit_[ticks]</t>
     </r>
     <r>
@@ -222,16 +228,45 @@
     <t>The UI or Backend blocks the submission and displays a validation error for the Name field.</t>
   </si>
   <si>
-    <t>UI failed to display an error message when the Name field was left empty.</t>
-  </si>
-  <si>
-    <t>FAILED</t>
+    <t>The browser's native HTML5 validation blocked the form submission and displayed a 'Please fill out this field' warning.</t>
+  </si>
+  <si>
+    <t>PASS</t>
   </si>
   <si>
     <t>TC_CAT_02</t>
   </si>
   <si>
     <t>Verify creation with duplicate Category Name</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">User is on </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF444746"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>.../Admin/Categories/Create</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>.</t>
+    </r>
   </si>
   <si>
     <t>1. Create a Category successfully. 
@@ -246,9 +281,6 @@
     <t>Backend successfully blocked the duplicate name and showed an error.</t>
   </si>
   <si>
-    <t>PASS</t>
-  </si>
-  <si>
     <t>TC_CAT_03</t>
   </si>
   <si>
@@ -256,6 +288,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">1. Enter a valid Name. 
 2. Enter </t>
     </r>
@@ -296,6 +334,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">1. Navigate directly to </t>
     </r>
     <r>
@@ -334,6 +378,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">User is on </t>
     </r>
     <r>
@@ -357,6 +407,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>1. Enter a unique Unit Name and ShortName (</t>
     </r>
     <r>
@@ -393,6 +449,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">User is on </t>
     </r>
     <r>
@@ -432,6 +494,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">1. Click the Edit button for a Unit. 
 2. Change ShortName to </t>
     </r>
@@ -488,6 +556,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">User is on </t>
     </r>
     <r>
@@ -545,6 +619,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">1. Enter </t>
     </r>
     <r>
@@ -581,6 +661,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">1. Navigate directly to </t>
     </r>
     <r>
@@ -614,12 +700,12 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -647,13 +733,7 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -662,22 +742,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -692,17 +757,31 @@
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF9C6500"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -721,7 +800,21 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -730,17 +823,18 @@
     </font>
     <font>
       <b/>
-      <sz val="15"/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -760,6 +854,21 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF3F3F3F"/>
@@ -767,36 +876,6 @@
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="33">
     <fill>
@@ -807,187 +886,187 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1012,6 +1091,26 @@
       </top>
       <bottom style="medium">
         <color rgb="FF1F1F1F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1036,15 +1135,6 @@
       </top>
       <bottom style="thin">
         <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1081,11 +1171,9 @@
     <border>
       <left/>
       <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1104,175 +1192,160 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="16" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="14" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="13" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1614,47 +1687,47 @@
     <col min="3" max="3" width="80.8888888888889" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.55" spans="1:3">
-      <c r="A1" s="7" t="s">
+    <row r="1" ht="15.15" spans="1:3">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" ht="28.35" spans="1:3">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="6" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" ht="28.35" spans="1:3">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="6" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="4" ht="28.35" spans="1:3">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="6" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1676,7 +1749,7 @@
     <col min="4" max="4" width="58.3333333333333" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.55" spans="1:4">
+    <row r="1" ht="15.15" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
@@ -1690,14 +1763,14 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" ht="14.55" spans="1:4">
+    <row r="2" ht="15.15" spans="1:4">
       <c r="A2" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D2" s="2" t="s">
@@ -1711,21 +1784,21 @@
       <c r="B3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="4" t="s">
         <v>22</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="4" ht="14.55" spans="1:4">
+    <row r="4" ht="15.15" spans="1:4">
       <c r="A4" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="4">
         <v>9999999</v>
       </c>
       <c r="D4" s="2" t="s">
@@ -1739,49 +1812,49 @@
       <c r="B5" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="4" t="s">
         <v>29</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="6" ht="14.55" spans="1:4">
+    <row r="6" ht="15.15" spans="1:4">
       <c r="A6" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="4" t="s">
         <v>33</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="7" ht="14.55" spans="1:4">
+    <row r="7" ht="15.15" spans="1:4">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="8" ht="14.55" spans="1:4">
+    <row r="8" ht="15.15" spans="1:4">
       <c r="A8" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="4" t="s">
         <v>38</v>
       </c>
       <c r="D8" s="2" t="s">
@@ -1810,7 +1883,7 @@
     <col min="8" max="8" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.55" spans="1:8">
+    <row r="1" ht="15.15" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>40</v>
       </c>
@@ -1858,7 +1931,7 @@
       <c r="G2" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="2" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1873,19 +1946,19 @@
         <v>57</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" ht="55.95" spans="1:8">
@@ -1899,9 +1972,9 @@
         <v>63</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E4" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>64</v>
       </c>
       <c r="F4" s="3" t="s">
@@ -1911,7 +1984,7 @@
         <v>66</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" ht="28.35" spans="1:8">
@@ -1937,7 +2010,7 @@
         <v>72</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6" ht="28.35" spans="1:8">
@@ -1953,7 +2026,7 @@
       <c r="D6" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="3" t="s">
         <v>77</v>
       </c>
       <c r="F6" s="3" t="s">
@@ -1963,7 +2036,7 @@
         <v>79</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" ht="42.15" spans="1:8">
@@ -1989,7 +2062,7 @@
         <v>85</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8" ht="42.15" spans="1:8">
@@ -2005,7 +2078,7 @@
       <c r="D8" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="3" t="s">
         <v>88</v>
       </c>
       <c r="F8" s="3" t="s">
@@ -2015,7 +2088,7 @@
         <v>90</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" ht="28.35" spans="1:8">
@@ -2041,7 +2114,7 @@
         <v>95</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" ht="28.35" spans="1:8">
@@ -2067,7 +2140,7 @@
         <v>102</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" ht="55.95" spans="1:8">
@@ -2093,7 +2166,7 @@
         <v>107</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" ht="42.15" spans="1:8">
@@ -2109,7 +2182,7 @@
       <c r="D12" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="3" t="s">
         <v>110</v>
       </c>
       <c r="F12" s="3" t="s">
@@ -2119,7 +2192,7 @@
         <v>112</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" ht="28.35" spans="1:8">
@@ -2145,7 +2218,7 @@
         <v>117</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>